<commit_message>
docs(lab4): expand AI review and defect analysis
</commit_message>
<xml_diff>
--- a/实验四_软件质量工程与AI辅助代码审查/D4-6_缺陷台账与缺陷分析会纪要.xlsx
+++ b/实验四_软件质量工程与AI辅助代码审查/D4-6_缺陷台账与缺陷分析会纪要.xlsx
@@ -10,11 +10,17 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="缺陷台账" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="度量指标" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bug Bash 纪要" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="四象限排序" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'缺陷台账'!$A$1:$O$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'度量指标'!$A$1:$E$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Bug Bash 纪要'!$A$1:$B$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'缺陷台账'!$A$1:$S$17</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'缺陷台账'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'度量指标'!$A$1:$E$12</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'度量指标'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Bug Bash 纪要'!$A$1:$B$17</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Bug Bash 纪要'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'四象限排序'!$A$1:$D$5</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">'四象限排序'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -23,7 +29,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -44,8 +50,13 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -67,8 +78,38 @@
         <fgColor rgb="00D9EAF7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000B6B3A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4CCCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAD3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2F0D9"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -90,11 +131,25 @@
         <color rgb="00B8D8C2"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B7C9BD"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B7C9BD"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B7C9BD"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B7C9BD"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -115,6 +170,30 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -480,1032 +559,1677 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O13"/>
+  <dimension ref="A1:S17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
     <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="34" customWidth="1" min="16" max="16"/>
+    <col width="30" customWidth="1" min="17" max="17"/>
+    <col width="22" customWidth="1" min="18" max="18"/>
+    <col width="20" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="4" t="inlineStr">
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>缺陷ID</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="8" t="inlineStr">
         <is>
           <t>标题</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="8" t="inlineStr">
         <is>
           <t>严重度(S1-S4)</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="8" t="inlineStr">
         <is>
           <t>优先级(P0-P3)</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="8" t="inlineStr">
         <is>
           <t>模块</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="F1" s="8" t="inlineStr">
         <is>
           <t>发现阶段</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G1" s="8" t="inlineStr">
         <is>
           <t>发现方式</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="H1" s="8" t="inlineStr">
         <is>
           <t>报告人</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="I1" s="8" t="inlineStr">
         <is>
           <t>处理人</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="J1" s="8" t="inlineStr">
         <is>
           <t>状态</t>
         </is>
       </c>
-      <c r="K1" s="4" t="inlineStr">
+      <c r="K1" s="8" t="inlineStr">
         <is>
           <t>创建时间</t>
         </is>
       </c>
-      <c r="L1" s="4" t="inlineStr">
+      <c r="L1" s="8" t="inlineStr">
         <is>
           <t>关闭时间</t>
         </is>
       </c>
-      <c r="M1" s="4" t="inlineStr">
+      <c r="M1" s="8" t="inlineStr">
         <is>
           <t>修复 PR</t>
         </is>
       </c>
-      <c r="N1" s="4" t="inlineStr">
+      <c r="N1" s="8" t="inlineStr">
         <is>
           <t>根因分类</t>
         </is>
       </c>
-      <c r="O1" s="4" t="inlineStr">
+      <c r="O1" s="8" t="inlineStr">
+        <is>
+          <t>影响范围</t>
+        </is>
+      </c>
+      <c r="P1" s="8" t="inlineStr">
+        <is>
+          <t>复现步骤</t>
+        </is>
+      </c>
+      <c r="Q1" s="8" t="inlineStr">
+        <is>
+          <t>回归验证</t>
+        </is>
+      </c>
+      <c r="R1" s="8" t="inlineStr">
+        <is>
+          <t>关闭依据</t>
+        </is>
+      </c>
+      <c r="S1" s="8" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="5" t="inlineStr">
+    <row r="2" ht="50" customHeight="1">
+      <c r="A2" s="9" t="inlineStr">
         <is>
           <t>BUG-001</t>
         </is>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B2" s="9" t="inlineStr">
         <is>
           <t>橘猫预约被识别成橘子套餐</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C2" s="10" t="inlineStr">
         <is>
           <t>S2</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="D2" s="11" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="E2" s="9" t="inlineStr">
         <is>
           <t>推荐服务</t>
         </is>
       </c>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="F2" s="9" t="inlineStr">
         <is>
           <t>生产</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="G2" s="9" t="inlineStr">
         <is>
           <t>用户反馈</t>
         </is>
       </c>
-      <c r="H2" s="5" t="inlineStr">
-        <is>
-          <t>戴正宇</t>
-        </is>
-      </c>
-      <c r="I2" s="5" t="inlineStr">
-        <is>
-          <t>戴正宇</t>
-        </is>
-      </c>
-      <c r="J2" s="5" t="inlineStr">
+      <c r="H2" s="9" t="inlineStr">
+        <is>
+          <t>戴正宇</t>
+        </is>
+      </c>
+      <c r="I2" s="9" t="inlineStr">
+        <is>
+          <t>戴正宇</t>
+        </is>
+      </c>
+      <c r="J2" s="12" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="K2" s="5" t="inlineStr">
+      <c r="K2" s="9" t="inlineStr">
         <is>
           <t>2026-05-01</t>
         </is>
       </c>
-      <c r="L2" s="5" t="inlineStr">
+      <c r="L2" s="9" t="inlineStr">
         <is>
           <t>2026-05-02</t>
         </is>
       </c>
-      <c r="M2" s="5" t="inlineStr">
+      <c r="M2" s="9" t="inlineStr">
         <is>
           <t>PR-401</t>
         </is>
       </c>
-      <c r="N2" s="5" t="inlineStr">
+      <c r="N2" s="9" t="inlineStr">
         <is>
           <t>语义混淆</t>
         </is>
       </c>
-      <c r="O2" s="5" t="inlineStr">
-        <is>
-          <t>新增属性测试</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="O2" s="9" t="inlineStr">
+        <is>
+          <t>AI 推荐与套餐映射</t>
+        </is>
+      </c>
+      <c r="P2" s="9" t="inlineStr">
+        <is>
+          <t>输入“橘猫陪伴预约”后查看推荐 SKU</t>
+        </is>
+      </c>
+      <c r="Q2" s="9" t="inlineStr">
+        <is>
+          <t>属性测试 test_orange_cat_semantics_are_stable</t>
+        </is>
+      </c>
+      <c r="R2" s="9" t="inlineStr">
+        <is>
+          <t>D4-3 测试全绿</t>
+        </is>
+      </c>
+      <c r="S2" s="9" t="inlineStr">
+        <is>
+          <t>历史牵引缺陷</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="50" customHeight="1">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>BUG-002</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
         <is>
           <t>预约人数为 0 时仍返回成功</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="10" t="inlineStr">
         <is>
           <t>S2</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="11" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E3" s="9" t="inlineStr">
         <is>
           <t>预约服务</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F3" s="9" t="inlineStr">
         <is>
           <t>单元测试</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="G3" s="9" t="inlineStr">
         <is>
           <t>自动化</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
-        <is>
-          <t>戴正宇</t>
-        </is>
-      </c>
-      <c r="I3" s="5" t="inlineStr">
-        <is>
-          <t>戴正宇</t>
-        </is>
-      </c>
-      <c r="J3" s="5" t="inlineStr">
+      <c r="H3" s="9" t="inlineStr">
+        <is>
+          <t>戴正宇</t>
+        </is>
+      </c>
+      <c r="I3" s="9" t="inlineStr">
+        <is>
+          <t>戴正宇</t>
+        </is>
+      </c>
+      <c r="J3" s="12" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="K3" s="5" t="inlineStr">
+      <c r="K3" s="9" t="inlineStr">
         <is>
           <t>2026-05-02</t>
         </is>
       </c>
-      <c r="L3" s="5" t="inlineStr">
+      <c r="L3" s="9" t="inlineStr">
         <is>
           <t>2026-05-02</t>
         </is>
       </c>
-      <c r="M3" s="5" t="inlineStr">
+      <c r="M3" s="9" t="inlineStr">
         <is>
           <t>PR-401</t>
         </is>
       </c>
-      <c r="N3" s="5" t="inlineStr">
+      <c r="N3" s="9" t="inlineStr">
         <is>
           <t>边界遗漏</t>
         </is>
       </c>
-      <c r="O3" s="5" t="inlineStr">
+      <c r="O3" s="9" t="inlineStr">
+        <is>
+          <t>预约容量校验</t>
+        </is>
+      </c>
+      <c r="P3" s="9" t="inlineStr">
+        <is>
+          <t>partySize=0 调用创建预约</t>
+        </is>
+      </c>
+      <c r="Q3" s="9" t="inlineStr">
+        <is>
+          <t>unit/test_zero_party_size_rejected</t>
+        </is>
+      </c>
+      <c r="R3" s="9" t="inlineStr">
+        <is>
+          <t>边界用例通过</t>
+        </is>
+      </c>
+      <c r="S3" s="9" t="inlineStr">
         <is>
           <t>validate_party_size</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+    <row r="4" ht="50" customHeight="1">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>BUG-003</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>取消已取消预约未返回幂等结果</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="13" t="inlineStr">
         <is>
           <t>S3</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="10" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="9" t="inlineStr">
         <is>
           <t>预约服务</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="9" t="inlineStr">
         <is>
           <t>集成测试</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G4" s="9" t="inlineStr">
         <is>
           <t>自动化</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>戴正宇</t>
-        </is>
-      </c>
-      <c r="I4" s="5" t="inlineStr">
-        <is>
-          <t>戴正宇</t>
-        </is>
-      </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>戴正宇</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>戴正宇</t>
+        </is>
+      </c>
+      <c r="J4" s="12" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr">
+      <c r="K4" s="9" t="inlineStr">
         <is>
           <t>2026-05-03</t>
         </is>
       </c>
-      <c r="L4" s="5" t="inlineStr">
+      <c r="L4" s="9" t="inlineStr">
         <is>
           <t>2026-05-03</t>
         </is>
       </c>
-      <c r="M4" s="5" t="inlineStr">
+      <c r="M4" s="9" t="inlineStr">
         <is>
           <t>PR-401</t>
         </is>
       </c>
-      <c r="N4" s="5" t="inlineStr">
+      <c r="N4" s="9" t="inlineStr">
         <is>
           <t>状态迁移遗漏</t>
         </is>
       </c>
-      <c r="O4" s="5" t="inlineStr">
+      <c r="O4" s="9" t="inlineStr">
+        <is>
+          <t>取消流程和桌位释放</t>
+        </is>
+      </c>
+      <c r="P4" s="9" t="inlineStr">
+        <is>
+          <t>对同一 reservationId 连续取消两次</t>
+        </is>
+      </c>
+      <c r="Q4" s="9" t="inlineStr">
+        <is>
+          <t>integration/test_cancelled_reservation_is_idempotent</t>
+        </is>
+      </c>
+      <c r="R4" s="9" t="inlineStr">
+        <is>
+          <t>状态机回归通过</t>
+        </is>
+      </c>
+      <c r="S4" s="9" t="inlineStr">
         <is>
           <t>补状态测试</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+    <row r="5" ht="50" customHeight="1">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>BUG-004</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>会员手机号在日志中明文输出</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="10" t="inlineStr">
         <is>
           <t>S2</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="11" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E5" s="9" t="inlineStr">
         <is>
           <t>会员服务</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="F5" s="9" t="inlineStr">
         <is>
           <t>AI Review</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>人工审查</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>戴正宇</t>
-        </is>
-      </c>
-      <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>戴正宇</t>
-        </is>
-      </c>
-      <c r="J5" s="5" t="inlineStr">
+      <c r="H5" s="9" t="inlineStr">
+        <is>
+          <t>戴正宇</t>
+        </is>
+      </c>
+      <c r="I5" s="9" t="inlineStr">
+        <is>
+          <t>戴正宇</t>
+        </is>
+      </c>
+      <c r="J5" s="12" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="K5" s="5" t="inlineStr">
+      <c r="K5" s="9" t="inlineStr">
         <is>
           <t>2026-05-03</t>
         </is>
       </c>
-      <c r="L5" s="5" t="inlineStr">
+      <c r="L5" s="9" t="inlineStr">
         <is>
           <t>2026-05-04</t>
         </is>
       </c>
-      <c r="M5" s="5" t="inlineStr">
+      <c r="M5" s="9" t="inlineStr">
         <is>
           <t>PR-402</t>
         </is>
       </c>
-      <c r="N5" s="5" t="inlineStr">
+      <c r="N5" s="9" t="inlineStr">
         <is>
           <t>隐私脱敏</t>
         </is>
       </c>
-      <c r="O5" s="5" t="inlineStr">
+      <c r="O5" s="9" t="inlineStr">
+        <is>
+          <t>日志、截图、HTML 报告</t>
+        </is>
+      </c>
+      <c r="P5" s="9" t="inlineStr">
+        <is>
+          <t>触发会员资料异常后检查日志</t>
+        </is>
+      </c>
+      <c r="Q5" s="9" t="inlineStr">
+        <is>
+          <t>unit/test_privacy_helpers</t>
+        </is>
+      </c>
+      <c r="R5" s="9" t="inlineStr">
+        <is>
+          <t>日志抽样无完整手机号</t>
+        </is>
+      </c>
+      <c r="S5" s="9" t="inlineStr">
         <is>
           <t>mask_phone</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+    <row r="6" ht="50" customHeight="1">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>BUG-005</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>预约备注可注入脚本片段</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="10" t="inlineStr">
         <is>
           <t>S2</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="10" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="9" t="inlineStr">
         <is>
           <t>预约服务</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F6" s="9" t="inlineStr">
         <is>
           <t>安全测试</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>ZAP 规则</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>戴正宇</t>
-        </is>
-      </c>
-      <c r="I6" s="5" t="inlineStr">
-        <is>
-          <t>戴正宇</t>
-        </is>
-      </c>
-      <c r="J6" s="5" t="inlineStr">
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>戴正宇</t>
+        </is>
+      </c>
+      <c r="I6" s="9" t="inlineStr">
+        <is>
+          <t>戴正宇</t>
+        </is>
+      </c>
+      <c r="J6" s="12" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="K6" s="5" t="inlineStr">
+      <c r="K6" s="9" t="inlineStr">
         <is>
           <t>2026-05-04</t>
         </is>
       </c>
-      <c r="L6" s="5" t="inlineStr">
+      <c r="L6" s="9" t="inlineStr">
         <is>
           <t>2026-05-04</t>
         </is>
       </c>
-      <c r="M6" s="5" t="inlineStr">
+      <c r="M6" s="9" t="inlineStr">
         <is>
           <t>PR-402</t>
         </is>
       </c>
-      <c r="N6" s="5" t="inlineStr">
+      <c r="N6" s="9" t="inlineStr">
         <is>
           <t>输入未转义</t>
         </is>
       </c>
-      <c r="O6" s="5" t="inlineStr">
+      <c r="O6" s="9" t="inlineStr">
+        <is>
+          <t>预约备注和评价内容</t>
+        </is>
+      </c>
+      <c r="P6" s="9" t="inlineStr">
+        <is>
+          <t>备注输入 &lt;script&gt;alert(1)&lt;/script&gt;</t>
+        </is>
+      </c>
+      <c r="Q6" s="9" t="inlineStr">
+        <is>
+          <t>unit/property sanitize_note</t>
+        </is>
+      </c>
+      <c r="R6" s="9" t="inlineStr">
+        <is>
+          <t>HTML 转义断言通过</t>
+        </is>
+      </c>
+      <c r="S6" s="9" t="inlineStr">
         <is>
           <t>sanitize_note</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+    <row r="7" ht="50" customHeight="1">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>BUG-006</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>契约测试只覆盖成功路径</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" s="13" t="inlineStr">
         <is>
           <t>S3</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D7" s="10" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E7" s="9" t="inlineStr">
         <is>
           <t>契约</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="F7" s="9" t="inlineStr">
         <is>
           <t>AI Review</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>人工审查</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>戴正宇</t>
-        </is>
-      </c>
-      <c r="I7" s="5" t="inlineStr">
-        <is>
-          <t>戴正宇</t>
-        </is>
-      </c>
-      <c r="J7" s="5" t="inlineStr">
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>戴正宇</t>
+        </is>
+      </c>
+      <c r="I7" s="9" t="inlineStr">
+        <is>
+          <t>戴正宇</t>
+        </is>
+      </c>
+      <c r="J7" s="12" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="K7" s="5" t="inlineStr">
+      <c r="K7" s="9" t="inlineStr">
         <is>
           <t>2026-05-04</t>
         </is>
       </c>
-      <c r="L7" s="5" t="inlineStr">
+      <c r="L7" s="9" t="inlineStr">
         <is>
           <t>2026-05-05</t>
         </is>
       </c>
-      <c r="M7" s="5" t="inlineStr">
+      <c r="M7" s="9" t="inlineStr">
         <is>
           <t>PR-401</t>
         </is>
       </c>
-      <c r="N7" s="5" t="inlineStr">
+      <c r="N7" s="9" t="inlineStr">
         <is>
           <t>测试覆盖不足</t>
         </is>
       </c>
-      <c r="O7" s="5" t="inlineStr">
+      <c r="O7" s="9" t="inlineStr">
+        <is>
+          <t>消费者错误处理</t>
+        </is>
+      </c>
+      <c r="P7" s="9" t="inlineStr">
+        <is>
+          <t>检查 contract JSON 是否含 error_schema</t>
+        </is>
+      </c>
+      <c r="Q7" s="9" t="inlineStr">
+        <is>
+          <t>contract/test_error_schema_is_uniform</t>
+        </is>
+      </c>
+      <c r="R7" s="9" t="inlineStr">
+        <is>
+          <t>契约断言通过</t>
+        </is>
+      </c>
+      <c r="S7" s="9" t="inlineStr">
         <is>
           <t>补 error_schema</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+    <row r="8" ht="50" customHeight="1">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>BUG-007</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>测试报告未输出机器可读 JSON</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="14" t="inlineStr">
         <is>
           <t>S4</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="13" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E8" s="9" t="inlineStr">
         <is>
           <t>质量工具</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="F8" s="9" t="inlineStr">
         <is>
           <t>自测</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="G8" s="9" t="inlineStr">
         <is>
           <t>人工审查</t>
         </is>
       </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>戴正宇</t>
-        </is>
-      </c>
-      <c r="I8" s="5" t="inlineStr">
-        <is>
-          <t>戴正宇</t>
-        </is>
-      </c>
-      <c r="J8" s="5" t="inlineStr">
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>戴正宇</t>
+        </is>
+      </c>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>戴正宇</t>
+        </is>
+      </c>
+      <c r="J8" s="12" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="K8" s="5" t="inlineStr">
+      <c r="K8" s="9" t="inlineStr">
         <is>
           <t>2026-05-05</t>
         </is>
       </c>
-      <c r="L8" s="5" t="inlineStr">
+      <c r="L8" s="9" t="inlineStr">
         <is>
           <t>2026-05-05</t>
         </is>
       </c>
-      <c r="M8" s="5" t="inlineStr">
+      <c r="M8" s="9" t="inlineStr">
         <is>
           <t>PR-402</t>
         </is>
       </c>
-      <c r="N8" s="5" t="inlineStr">
+      <c r="N8" s="9" t="inlineStr">
         <is>
           <t>可审计性不足</t>
         </is>
       </c>
-      <c r="O8" s="5" t="inlineStr">
+      <c r="O8" s="9" t="inlineStr">
+        <is>
+          <t>CI 质量看板</t>
+        </is>
+      </c>
+      <c r="P8" s="9" t="inlineStr">
+        <is>
+          <t>运行 run_tests.py 后检查 reports 目录</t>
+        </is>
+      </c>
+      <c r="Q8" s="9" t="inlineStr">
+        <is>
+          <t>test-results.json 已生成</t>
+        </is>
+      </c>
+      <c r="R8" s="9" t="inlineStr">
+        <is>
+          <t>D4-3 JSON 存在</t>
+        </is>
+      </c>
+      <c r="S8" s="9" t="inlineStr">
         <is>
           <t>新增 test-results.json</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+    <row r="9" ht="50" customHeight="1">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>BUG-008</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>E2E 旅程与 RTM 不可追溯</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" s="13" t="inlineStr">
         <is>
           <t>S3</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="10" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E9" s="9" t="inlineStr">
         <is>
           <t>测试管理</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="F9" s="9" t="inlineStr">
         <is>
           <t>文档审查</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="G9" s="9" t="inlineStr">
         <is>
           <t>人工审查</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>戴正宇</t>
-        </is>
-      </c>
-      <c r="I9" s="5" t="inlineStr">
-        <is>
-          <t>戴正宇</t>
-        </is>
-      </c>
-      <c r="J9" s="5" t="inlineStr">
+      <c r="H9" s="9" t="inlineStr">
+        <is>
+          <t>戴正宇</t>
+        </is>
+      </c>
+      <c r="I9" s="9" t="inlineStr">
+        <is>
+          <t>戴正宇</t>
+        </is>
+      </c>
+      <c r="J9" s="12" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="K9" s="5" t="inlineStr">
+      <c r="K9" s="9" t="inlineStr">
         <is>
           <t>2026-05-05</t>
         </is>
       </c>
-      <c r="L9" s="5" t="inlineStr">
+      <c r="L9" s="9" t="inlineStr">
         <is>
           <t>2026-05-06</t>
         </is>
       </c>
-      <c r="M9" s="5" t="inlineStr">
+      <c r="M9" s="9" t="inlineStr">
         <is>
           <t>PR-403</t>
         </is>
       </c>
-      <c r="N9" s="5" t="inlineStr">
+      <c r="N9" s="9" t="inlineStr">
         <is>
           <t>追溯缺失</t>
         </is>
       </c>
-      <c r="O9" s="5" t="inlineStr">
+      <c r="O9" s="9" t="inlineStr">
+        <is>
+          <t>需求验收与答辩审计</t>
+        </is>
+      </c>
+      <c r="P9" s="9" t="inlineStr">
+        <is>
+          <t>抽查 E2E 用例是否绑定 FR</t>
+        </is>
+      </c>
+      <c r="Q9" s="9" t="inlineStr">
+        <is>
+          <t>D4-2/D4-8 追溯检查</t>
+        </is>
+      </c>
+      <c r="R9" s="9" t="inlineStr">
+        <is>
+          <t>RTM 已补充</t>
+        </is>
+      </c>
+      <c r="S9" s="9" t="inlineStr">
         <is>
           <t>补 D4-8</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+    <row r="10" ht="50" customHeight="1">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>BUG-009</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>闭店时段仍可生成预约</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C10" s="10" t="inlineStr">
         <is>
           <t>S2</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D10" s="10" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E10" s="9" t="inlineStr">
         <is>
           <t>配置服务</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="F10" s="9" t="inlineStr">
         <is>
           <t>集成测试</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="G10" s="9" t="inlineStr">
         <is>
           <t>自动化</t>
         </is>
       </c>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>戴正宇</t>
-        </is>
-      </c>
-      <c r="I10" s="5" t="inlineStr">
-        <is>
-          <t>戴正宇</t>
-        </is>
-      </c>
-      <c r="J10" s="5" t="inlineStr">
+      <c r="H10" s="9" t="inlineStr">
+        <is>
+          <t>戴正宇</t>
+        </is>
+      </c>
+      <c r="I10" s="9" t="inlineStr">
+        <is>
+          <t>戴正宇</t>
+        </is>
+      </c>
+      <c r="J10" s="12" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="K10" s="5" t="inlineStr">
+      <c r="K10" s="9" t="inlineStr">
         <is>
           <t>2026-05-06</t>
         </is>
       </c>
-      <c r="L10" s="5" t="inlineStr">
+      <c r="L10" s="9" t="inlineStr">
         <is>
           <t>2026-05-06</t>
         </is>
       </c>
-      <c r="M10" s="5" t="inlineStr">
+      <c r="M10" s="9" t="inlineStr">
         <is>
           <t>PR-401</t>
         </is>
       </c>
-      <c r="N10" s="5" t="inlineStr">
+      <c r="N10" s="9" t="inlineStr">
         <is>
           <t>业务规则遗漏</t>
         </is>
       </c>
-      <c r="O10" s="5" t="inlineStr">
+      <c r="O10" s="9" t="inlineStr">
+        <is>
+          <t>门店配置与预约入口</t>
+        </is>
+      </c>
+      <c r="P10" s="9" t="inlineStr">
+        <is>
+          <t>配置闭店时段后创建预约</t>
+        </is>
+      </c>
+      <c r="Q10" s="9" t="inlineStr">
+        <is>
+          <t>D4-2 TC-057/TC-058</t>
+        </is>
+      </c>
+      <c r="R10" s="9" t="inlineStr">
+        <is>
+          <t>配置用例通过</t>
+        </is>
+      </c>
+      <c r="S10" s="9" t="inlineStr">
         <is>
           <t>补配置测试</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+    <row r="11" ht="50" customHeight="1">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>BUG-010</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>质量门禁未声明变异分数阈值</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C11" s="14" t="inlineStr">
         <is>
           <t>S4</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D11" s="13" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="E11" s="9" t="inlineStr">
         <is>
           <t>CI/CD</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="F11" s="9" t="inlineStr">
         <is>
           <t>文档审查</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr">
+      <c r="G11" s="9" t="inlineStr">
         <is>
           <t>AI Review</t>
         </is>
       </c>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>戴正宇</t>
-        </is>
-      </c>
-      <c r="I11" s="5" t="inlineStr">
-        <is>
-          <t>戴正宇</t>
-        </is>
-      </c>
-      <c r="J11" s="5" t="inlineStr">
+      <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t>戴正宇</t>
+        </is>
+      </c>
+      <c r="I11" s="9" t="inlineStr">
+        <is>
+          <t>戴正宇</t>
+        </is>
+      </c>
+      <c r="J11" s="12" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="K11" s="5" t="inlineStr">
+      <c r="K11" s="9" t="inlineStr">
         <is>
           <t>2026-05-06</t>
         </is>
       </c>
-      <c r="L11" s="5" t="inlineStr">
+      <c r="L11" s="9" t="inlineStr">
         <is>
           <t>2026-05-06</t>
         </is>
       </c>
-      <c r="M11" s="5" t="inlineStr">
+      <c r="M11" s="9" t="inlineStr">
         <is>
           <t>PR-403</t>
         </is>
       </c>
-      <c r="N11" s="5" t="inlineStr">
+      <c r="N11" s="9" t="inlineStr">
         <is>
           <t>流程缺失</t>
         </is>
       </c>
-      <c r="O11" s="5" t="inlineStr">
+      <c r="O11" s="9" t="inlineStr">
+        <is>
+          <t>发布准出标准</t>
+        </is>
+      </c>
+      <c r="P11" s="9" t="inlineStr">
+        <is>
+          <t>检查 D4-1 是否列明 mutation 阈值</t>
+        </is>
+      </c>
+      <c r="Q11" s="9" t="inlineStr">
+        <is>
+          <t>D4-1/D4-3 指标一致</t>
+        </is>
+      </c>
+      <c r="R11" s="9" t="inlineStr">
+        <is>
+          <t>文档复核通过</t>
+        </is>
+      </c>
+      <c r="S11" s="9" t="inlineStr">
         <is>
           <t>补 D4-1</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+    <row r="12" ht="50" customHeight="1">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>BUG-011</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>中文深路径下测试工作目录不稳定</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C12" s="13" t="inlineStr">
         <is>
           <t>S3</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D12" s="13" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="E12" s="9" t="inlineStr">
         <is>
           <t>测试工具</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="F12" s="9" t="inlineStr">
         <is>
           <t>本地运行</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="G12" s="9" t="inlineStr">
         <is>
           <t>自动化</t>
         </is>
       </c>
-      <c r="H12" s="5" t="inlineStr">
-        <is>
-          <t>戴正宇</t>
-        </is>
-      </c>
-      <c r="I12" s="5" t="inlineStr">
-        <is>
-          <t>戴正宇</t>
-        </is>
-      </c>
-      <c r="J12" s="5" t="inlineStr">
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>戴正宇</t>
+        </is>
+      </c>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>戴正宇</t>
+        </is>
+      </c>
+      <c r="J12" s="12" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="K12" s="5" t="inlineStr">
+      <c r="K12" s="9" t="inlineStr">
         <is>
           <t>2026-05-07</t>
         </is>
       </c>
-      <c r="L12" s="5" t="inlineStr">
+      <c r="L12" s="9" t="inlineStr">
         <is>
           <t>2026-05-07</t>
         </is>
       </c>
-      <c r="M12" s="5" t="inlineStr">
+      <c r="M12" s="9" t="inlineStr">
         <is>
           <t>PR-402</t>
         </is>
       </c>
-      <c r="N12" s="5" t="inlineStr">
+      <c r="N12" s="9" t="inlineStr">
         <is>
           <t>环境兼容</t>
         </is>
       </c>
-      <c r="O12" s="5" t="inlineStr">
+      <c r="O12" s="9" t="inlineStr">
+        <is>
+          <t>Windows 本机执行</t>
+        </is>
+      </c>
+      <c r="P12" s="9" t="inlineStr">
+        <is>
+          <t>在中文路径运行渲染和测试命令</t>
+        </is>
+      </c>
+      <c r="Q12" s="9" t="inlineStr">
+        <is>
+          <t>英文临时目录规避验证</t>
+        </is>
+      </c>
+      <c r="R12" s="9" t="inlineStr">
+        <is>
+          <t>D4-4 渲染成功</t>
+        </is>
+      </c>
+      <c r="S12" s="9" t="inlineStr">
         <is>
           <t>从根目录运行</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+    <row r="13" ht="50" customHeight="1">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>BUG-012</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>模板隐藏占位符未被文本搜索发现</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C13" s="14" t="inlineStr">
         <is>
           <t>S4</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D13" s="13" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="E13" s="9" t="inlineStr">
         <is>
           <t>文档质量</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="F13" s="9" t="inlineStr">
         <is>
           <t>文档扫描</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr">
+      <c r="G13" s="9" t="inlineStr">
         <is>
           <t>自动化</t>
         </is>
       </c>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>戴正宇</t>
-        </is>
-      </c>
-      <c r="I13" s="5" t="inlineStr">
-        <is>
-          <t>戴正宇</t>
-        </is>
-      </c>
-      <c r="J13" s="5" t="inlineStr">
+      <c r="H13" s="9" t="inlineStr">
+        <is>
+          <t>戴正宇</t>
+        </is>
+      </c>
+      <c r="I13" s="9" t="inlineStr">
+        <is>
+          <t>戴正宇</t>
+        </is>
+      </c>
+      <c r="J13" s="12" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="K13" s="5" t="inlineStr">
+      <c r="K13" s="9" t="inlineStr">
         <is>
           <t>2026-05-07</t>
         </is>
       </c>
-      <c r="L13" s="5" t="inlineStr">
+      <c r="L13" s="9" t="inlineStr">
         <is>
           <t>2026-05-07</t>
         </is>
       </c>
-      <c r="M13" s="5" t="inlineStr">
+      <c r="M13" s="9" t="inlineStr">
         <is>
           <t>PR-403</t>
         </is>
       </c>
-      <c r="N13" s="5" t="inlineStr">
+      <c r="N13" s="9" t="inlineStr">
         <is>
           <t>审计遗漏</t>
         </is>
       </c>
-      <c r="O13" s="5" t="inlineStr">
+      <c r="O13" s="9" t="inlineStr">
+        <is>
+          <t>Word 表格与段落</t>
+        </is>
+      </c>
+      <c r="P13" s="9" t="inlineStr">
+        <is>
+          <t>普通 grep 搜索占位符</t>
+        </is>
+      </c>
+      <c r="Q13" s="9" t="inlineStr">
+        <is>
+          <t>python-docx 表格扫描</t>
+        </is>
+      </c>
+      <c r="R13" s="9" t="inlineStr">
+        <is>
+          <t>占位符扫描为 none</t>
+        </is>
+      </c>
+      <c r="S13" s="9" t="inlineStr">
         <is>
           <t>python-docx 扫描</t>
         </is>
       </c>
     </row>
+    <row r="14" ht="50" customHeight="1">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>BUG-013</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>押金非负保护变异体存活</t>
+        </is>
+      </c>
+      <c r="C14" s="13" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="D14" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>预约服务</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>变异测试</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t>mutation_check</t>
+        </is>
+      </c>
+      <c r="H14" s="9" t="inlineStr">
+        <is>
+          <t>戴正宇</t>
+        </is>
+      </c>
+      <c r="I14" s="9" t="inlineStr">
+        <is>
+          <t>戴正宇</t>
+        </is>
+      </c>
+      <c r="J14" s="15" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+      <c r="K14" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="L14" s="9" t="inlineStr"/>
+      <c r="M14" s="9" t="inlineStr">
+        <is>
+          <t>PR-404</t>
+        </is>
+      </c>
+      <c r="N14" s="9" t="inlineStr">
+        <is>
+          <t>断言强度不足</t>
+        </is>
+      </c>
+      <c r="O14" s="9" t="inlineStr">
+        <is>
+          <t>押金报价边界</t>
+        </is>
+      </c>
+      <c r="P14" s="9" t="inlineStr">
+        <is>
+          <t>删除 quote_deposit 非负保护后运行变异样本</t>
+        </is>
+      </c>
+      <c r="Q14" s="9" t="inlineStr">
+        <is>
+          <t>新增负数输入属性测试待补</t>
+        </is>
+      </c>
+      <c r="R14" s="9" t="inlineStr">
+        <is>
+          <t>纳入下轮补强</t>
+        </is>
+      </c>
+      <c r="S14" s="9" t="inlineStr">
+        <is>
+          <t>MUT-007</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="50" customHeight="1">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>BUG-014</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>预约表单缺少显式 label</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>前端页面</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>可访问性测试</t>
+        </is>
+      </c>
+      <c r="G15" s="9" t="inlineStr">
+        <is>
+          <t>Lighthouse/axe</t>
+        </is>
+      </c>
+      <c r="H15" s="9" t="inlineStr">
+        <is>
+          <t>戴正宇</t>
+        </is>
+      </c>
+      <c r="I15" s="9" t="inlineStr">
+        <is>
+          <t>戴正宇</t>
+        </is>
+      </c>
+      <c r="J15" s="12" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="K15" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="L15" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="M15" s="9" t="inlineStr">
+        <is>
+          <t>PR-404</t>
+        </is>
+      </c>
+      <c r="N15" s="9" t="inlineStr">
+        <is>
+          <t>可访问性遗漏</t>
+        </is>
+      </c>
+      <c r="O15" s="9" t="inlineStr">
+        <is>
+          <t>预约确认页</t>
+        </is>
+      </c>
+      <c r="P15" s="9" t="inlineStr">
+        <is>
+          <t>仅键盘填写预约表单并检查读屏标签</t>
+        </is>
+      </c>
+      <c r="Q15" s="9" t="inlineStr">
+        <is>
+          <t>D4-4 图4-7 对比</t>
+        </is>
+      </c>
+      <c r="R15" s="9" t="inlineStr">
+        <is>
+          <t>Accessibility 94</t>
+        </is>
+      </c>
+      <c r="S15" s="9" t="inlineStr">
+        <is>
+          <t>补 label/focus</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="50" customHeight="1">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>BUG-015</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>测试环境缺少严格 CSP</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>API 网关</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>安全测试</t>
+        </is>
+      </c>
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t>ZAP Baseline</t>
+        </is>
+      </c>
+      <c r="H16" s="9" t="inlineStr">
+        <is>
+          <t>戴正宇</t>
+        </is>
+      </c>
+      <c r="I16" s="9" t="inlineStr">
+        <is>
+          <t>戴正宇</t>
+        </is>
+      </c>
+      <c r="J16" s="13" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="K16" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="L16" s="9" t="inlineStr"/>
+      <c r="M16" s="9" t="inlineStr">
+        <is>
+          <t>PR-405</t>
+        </is>
+      </c>
+      <c r="N16" s="9" t="inlineStr">
+        <is>
+          <t>安全头配置</t>
+        </is>
+      </c>
+      <c r="O16" s="9" t="inlineStr">
+        <is>
+          <t>前端脚本加载策略</t>
+        </is>
+      </c>
+      <c r="P16" s="9" t="inlineStr">
+        <is>
+          <t>运行 ZAP baseline 查看 CSP 告警</t>
+        </is>
+      </c>
+      <c r="Q16" s="9" t="inlineStr">
+        <is>
+          <t>staging 网关开启后复测</t>
+        </is>
+      </c>
+      <c r="R16" s="9" t="inlineStr">
+        <is>
+          <t>记录残余风险</t>
+        </is>
+      </c>
+      <c r="S16" s="9" t="inlineStr">
+        <is>
+          <t>Medium 风险</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="50" customHeight="1">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>BUG-016</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>非功能报告缺少实机复测说明</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="inlineStr">
+        <is>
+          <t>S4</t>
+        </is>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>文档质量</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>文档审查</t>
+        </is>
+      </c>
+      <c r="G17" s="9" t="inlineStr">
+        <is>
+          <t>人工审查</t>
+        </is>
+      </c>
+      <c r="H17" s="9" t="inlineStr">
+        <is>
+          <t>戴正宇</t>
+        </is>
+      </c>
+      <c r="I17" s="9" t="inlineStr">
+        <is>
+          <t>戴正宇</t>
+        </is>
+      </c>
+      <c r="J17" s="12" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="K17" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="L17" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="M17" s="9" t="inlineStr">
+        <is>
+          <t>PR-405</t>
+        </is>
+      </c>
+      <c r="N17" s="9" t="inlineStr">
+        <is>
+          <t>证据说明不足</t>
+        </is>
+      </c>
+      <c r="O17" s="9" t="inlineStr">
+        <is>
+          <t>D4-4 报告可信度</t>
+        </is>
+      </c>
+      <c r="P17" s="9" t="inlineStr">
+        <is>
+          <t>检查性能/安全/可访问性章节是否说明来源</t>
+        </is>
+      </c>
+      <c r="Q17" s="9" t="inlineStr">
+        <is>
+          <t>D4-4 已补残余风险</t>
+        </is>
+      </c>
+      <c r="R17" s="9" t="inlineStr">
+        <is>
+          <t>文档复核通过</t>
+        </is>
+      </c>
+      <c r="S17" s="9" t="inlineStr">
+        <is>
+          <t>补充诚实说明</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O13"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <autoFilter ref="A1:S17"/>
+  <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -1513,186 +2237,302 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="29" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="54" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="4" t="inlineStr">
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>指标</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="8" t="inlineStr">
         <is>
           <t>本次值</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="8" t="inlineStr">
         <is>
           <t>基线值</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="8" t="inlineStr">
         <is>
           <t>变化</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="8" t="inlineStr">
         <is>
           <t>说明</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="5" t="inlineStr">
+    <row r="2" ht="50" customHeight="1">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>缺陷总数</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="n">
+        <v>16</v>
+      </c>
+      <c r="C2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" s="9" t="inlineStr">
+        <is>
+          <t>新增 16</t>
+        </is>
+      </c>
+      <c r="E2" s="9" t="inlineStr">
+        <is>
+          <t>覆盖生产反馈、自动化、AI Review、安全、可访问性和文档审查</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="50" customHeight="1">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>缺陷密度 (Defects / KLOC)</t>
         </is>
       </c>
-      <c r="B2" s="5" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="C2" s="5" t="n">
+      <c r="B3" s="9" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="C3" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t>下降 1.1</t>
-        </is>
-      </c>
-      <c r="E2" s="5" t="inlineStr">
-        <is>
-          <t>按 PoC 约 3.1 KLOC、12 个有效缺陷估算</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>上升 0.2</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>按 PoC 约 3.1 KLOC、16 个有效缺陷估算；本轮主动测试发现更多问题</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="50" customHeight="1">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>缺陷逃逸率 (%)</t>
         </is>
       </c>
-      <c r="B3" s="5" t="n">
-        <v>7.7</v>
-      </c>
-      <c r="C3" s="5" t="n">
+      <c r="B4" s="9" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="C4" s="9" t="n">
         <v>12</v>
       </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>下降 4.3</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>生产反馈 1 个 / 总缺陷 13 个口径</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>下降 5.7</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>生产反馈 1 个 / 总缺陷 16 个口径</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="50" customHeight="1">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>总体关闭率 (%)</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="n">
+        <v>87.5</v>
+      </c>
+      <c r="C5" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>上升 27.5</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>14 个 Closed / 16 个缺陷；Accepted/Deferred 均有残余风险说明</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="50" customHeight="1">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>P0/P1 未关闭数</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>下降 3</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>发布门禁要求 P0/P1 未关闭数为 0；BUG-015 为 Accepted 风险但已有补偿控制</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="50" customHeight="1">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>平均修复时长 MTTR (h)</t>
         </is>
       </c>
-      <c r="B4" s="5" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="C4" s="5" t="n">
+      <c r="B7" s="9" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="C7" s="9" t="n">
         <v>14</v>
       </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>下降 5.5</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>按关闭缺陷平均值</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>P0/P1 未关闭数</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="n">
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>下降 5.9</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>按 Closed 缺陷创建到关闭平均估算</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="50" customHeight="1">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>自动化通过率 (%)</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="C8" s="9" t="n">
+        <v>92</v>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>上升 8</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>D4-3 报告 38/38</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="50" customHeight="1">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>行覆盖率 (%)</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="n">
+        <v>72.5</v>
+      </c>
+      <c r="C9" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="C5" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>下降 3</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>发布门禁要求为 0</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>自动化通过率 (%)</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="n">
-        <v>100</v>
-      </c>
-      <c r="C6" s="5" t="n">
-        <v>92</v>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>上升 8</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>D4-3 报告 38/38</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>D4-3 reports/test-results.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="50" customHeight="1">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>分支覆盖率 (%)</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="C10" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>D4-3 reports/test-results.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="50" customHeight="1">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>变异样本分数 (%)</t>
         </is>
       </c>
-      <c r="B7" s="5" t="n">
-        <v>77.8</v>
-      </c>
-      <c r="C7" s="5" t="n">
+      <c r="B11" s="9" t="n">
+        <v>88.90000000000001</v>
+      </c>
+      <c r="C11" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D11" s="9" t="inlineStr">
         <is>
           <t>新增</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>轻量变异检查，非全量 mutmut</t>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>9 个轻量变异样本杀死 8 个</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="50" customHeight="1">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>AI Review 工程采纳率 (%)</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="n">
+        <v>88.90000000000001</v>
+      </c>
+      <c r="C12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>D4-5 18 条建议中采纳或部分采纳 16 条</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E7"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <autoFilter ref="A1:E12"/>
+  <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -1700,149 +2540,354 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="82" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="4" t="inlineStr">
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>项目</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="8" t="inlineStr">
         <is>
           <t>内容</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="6" t="inlineStr">
+    <row r="2" ht="50" customHeight="1">
+      <c r="A2" s="9" t="inlineStr">
         <is>
           <t>时间</t>
         </is>
       </c>
-      <c r="B2" s="6" t="inlineStr">
-        <is>
-          <t>2026-05-14  19:00-21:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-05  19:00-21:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="50" customHeight="1">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>地点</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
-        <is>
-          <t>线上 / GitHub PR + 本地报告</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>线上 / GitHub PR + 本地报告 + Word/Excel 交付物复核</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="50" customHeight="1">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>参会人</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>戴正宇；AI Reviewer；质量负责人视角复核</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>戴正宇；AI Reviewer（架构/安全/性能）；质量负责人视角复核</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="50" customHeight="1">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>会议目标</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>复盘实验四质量缺陷，确认 P0/P1 是否关闭，给出根因聚类、四象限排序和后续改进措施</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="50" customHeight="1">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>议程</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>1. 复盘线上语义缺陷  2. 过堂 12 个缺陷  3. 聚类根因  4. 制定质量门禁  5. 明确补跑事项</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>1. 复盘橘猫语义缺陷  2. 过堂 16 个缺陷  3. 按严重度×优先级排序  4. 聚类根因  5. 制定质量门禁与改进措施</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="50" customHeight="1">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>Top 5 根因</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>边界值遗漏、语义混淆、隐私脱敏不足、契约覆盖不足、质量证据不可追溯</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
+    <row r="8" ht="50" customHeight="1">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>关键结论 1</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>P0/P1 缺陷已关闭或具备补偿控制，允许进入课程交付；P2/P3 残余风险进入下轮迭代</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="50" customHeight="1">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>关键结论 2</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>AI Review 对流程型和设计型问题发现有效，但对模板隐藏占位符、Windows 路径、表格交付格式存在漏报</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="50" customHeight="1">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>关键结论 3</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>性能、安全、可访问性报告必须明确“实机截图/报告图/可复现命令”的证据来源，避免混淆</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="50" customHeight="1">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>改进措施 1</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>新增属性测试模板；负责人戴正宇；截止 2026-05-14</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>新增属性测试模板，优先覆盖语义混淆、押金非负、容量单调性；负责人戴正宇；截止 2026-06-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="50" customHeight="1">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>改进措施 2</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>D4-8 强制需求-自动化测试追溯；负责人戴正宇；截止 2026-05-14</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>D4-8 强制需求-测试-缺陷-回归用例追溯；负责人戴正宇；截止 2026-06-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="50" customHeight="1">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>改进措施 3</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>AI Review 意见必须记录裁决；负责人戴正宇；截止 2026-05-14</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>AI Review 意见必须记录裁决和证据位置；负责人戴正宇；截止 2026-06-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="50" customHeight="1">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>改进措施 4</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>发布前补跑 k6/ZAP/axe；负责人戴正宇；截止 staging 可用后</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>staging 可用后补跑 k6/ZAP/axe，并替换 D4-4 中报告图；负责人戴正宇；截止 staging 可用后 1 天</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="50" customHeight="1">
+      <c r="A15" s="9" t="inlineStr">
         <is>
           <t>改进措施 5</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>CI 中保留 HTML 与 JSON 报告附件；负责人戴正宇；截止 2026-05-14</t>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>CI 中保留 HTML、JSON、覆盖率和变异测试报告附件；负责人戴正宇；截止 2026-06-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="50" customHeight="1">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>改进措施 6</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>文档交付前执行 python-docx/openpyxl 占位符扫描和 LibreOffice 导出抽查；负责人戴正宇；截止每次提交前</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="50" customHeight="1">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>会后跟踪</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>BUG-013 Deferred、BUG-015 Accepted 需在下次迭代复核；其余 Closed 缺陷保持回归用例</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B11"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <autoFilter ref="A1:B17"/>
+  <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>象限</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>判定规则</t>
+        </is>
+      </c>
+      <c r="C1" s="8" t="inlineStr">
+        <is>
+          <t>缺陷</t>
+        </is>
+      </c>
+      <c r="D1" s="8" t="inlineStr">
+        <is>
+          <t>处理策略</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="50" customHeight="1">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>Q1 立即修复</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>S1/S2 且 P0/P1</t>
+        </is>
+      </c>
+      <c r="C2" s="9" t="inlineStr">
+        <is>
+          <t>BUG-001, BUG-002, BUG-004, BUG-005, BUG-009</t>
+        </is>
+      </c>
+      <c r="D2" s="9" t="inlineStr">
+        <is>
+          <t>阻断发布；必须修复并回归</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="50" customHeight="1">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>Q2 计划修复</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>S3 且 P1/P2</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>BUG-003, BUG-006, BUG-008, BUG-011, BUG-013, BUG-014, BUG-015</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>进入当前或下一迭代；P1 需补偿控制</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="50" customHeight="1">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>Q3 流程改进</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>S4 且 P2/P3</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>BUG-007, BUG-010, BUG-012, BUG-016</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>通过文档、工具和门禁修复</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="50" customHeight="1">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>Q4 观察跟踪</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>低严重度且低优先级</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>暂无</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>保留观察，不影响本次交付</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D5"/>
+  <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>